<commit_message>
Modèle logique métier (#137)
* MAJ-modèle logique (#128) ba16b6d74c28099f6969d28439af1fce4ba38306
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-fr-lm-addendum.xlsx
+++ b/main/ig/StructureDefinition-fr-lm-addendum.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="116">
   <si>
     <t>Property</t>
   </si>
@@ -42,7 +42,7 @@
     <t>Title</t>
   </si>
   <si>
-    <t>Modèle logique métier - FR LM Addendum</t>
+    <t>Logical model - FR LM Addendum</t>
   </si>
   <si>
     <t>Status</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-05-15T08:08:15+00:00</t>
+    <t>2026-05-18T14:11:29+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -266,7 +266,7 @@
     <t>fr-lm-section.codeSection</t>
   </si>
   <si>
-    <t>fr-lm-addendum.titreSection</t>
+    <t>fr-lm-addendum.titleSection</t>
   </si>
   <si>
     <t xml:space="preserve">string
@@ -276,52 +276,99 @@
     <t>Titre de la section</t>
   </si>
   <si>
-    <t>fr-lm-section.titreSection</t>
-  </si>
-  <si>
-    <t>fr-lm-addendum.blocNarratif</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Narrative
-</t>
+    <t>fr-lm-section.titleSection</t>
+  </si>
+  <si>
+    <t>fr-lm-addendum.description</t>
   </si>
   <si>
     <t>Bloc narratif</t>
   </si>
   <si>
-    <t>fr-lm-section.blocNarratif</t>
-  </si>
-  <si>
-    <t>fr-lm-addendum.sousSection</t>
+    <t>fr-lm-section.description</t>
+  </si>
+  <si>
+    <t>fr-lm-addendum.author[x]</t>
   </si>
   <si>
     <t xml:space="preserve">Base
 </t>
   </si>
   <si>
+    <t>author[x] peut correspondre soit à un professionnel, soit à une organisation, soit à un système.</t>
+  </si>
+  <si>
+    <t>fr-lm-section.author[x]</t>
+  </si>
+  <si>
+    <t>fr-lm-addendum.author[x].authorProfessional</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-lm-health-professional
+</t>
+  </si>
+  <si>
+    <t>L'auteur est un professionnel de santé</t>
+  </si>
+  <si>
+    <t>fr-lm-section.author[x].authorProfessional</t>
+  </si>
+  <si>
+    <t>fr-lm-addendum.author[x].authorOrganisation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-lm-organisation
+</t>
+  </si>
+  <si>
+    <t>L'auteur est une organisation</t>
+  </si>
+  <si>
+    <t>fr-lm-section.author[x].authorOrganisation</t>
+  </si>
+  <si>
+    <t>fr-lm-addendum.author[x].authorDevice</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-lm-device
+</t>
+  </si>
+  <si>
+    <t>L'auteur est un système</t>
+  </si>
+  <si>
+    <t>fr-lm-section.author[x].authorDevice</t>
+  </si>
+  <si>
+    <t>fr-lm-addendum.informant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-lm-informant
+</t>
+  </si>
+  <si>
+    <t>Informateur</t>
+  </si>
+  <si>
+    <t>fr-lm-section.informant</t>
+  </si>
+  <si>
+    <t>fr-lm-addendum.subSection</t>
+  </si>
+  <si>
     <t>Sous-sections</t>
   </si>
   <si>
-    <t>fr-lm-section.sousSection</t>
-  </si>
-  <si>
-    <t>fr-lm-addendum.entree</t>
+    <t>fr-lm-section.subSection</t>
+  </si>
+  <si>
+    <t>fr-lm-addendum.entry</t>
   </si>
   <si>
     <t>Entrées</t>
   </si>
   <si>
-    <t>fr-lm-section.entree</t>
-  </si>
-  <si>
-    <t>fr-lm-addendum.auteur</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-lm-auteur
-</t>
-  </si>
-  <si>
-    <t>auteur du document</t>
+    <t>fr-lm-section.entry</t>
   </si>
 </sst>
 </file>
@@ -623,11 +670,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AJ8"/>
+  <dimension ref="A1:AJ12"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="23.7734375" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="23.7734375" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="37.2265625" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="37.2265625" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="10.8515625" customWidth="true" bestFit="true" hidden="true"/>
     <col min="4" max="4" width="7.6796875" customWidth="true" bestFit="true" hidden="true"/>
     <col min="5" max="5" width="5.80859375" customWidth="true" bestFit="true"/>
@@ -636,7 +683,7 @@
     <col min="8" max="8" width="13.953125" customWidth="true" bestFit="true"/>
     <col min="9" max="9" width="11.3671875" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="63.95703125" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="73.875" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>
@@ -657,7 +704,7 @@
     <col min="29" max="29" width="17.65625" customWidth="true" bestFit="true"/>
     <col min="30" max="30" width="14.7578125" customWidth="true" bestFit="true"/>
     <col min="31" max="31" width="12.359375" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="32" max="32" width="20.98828125" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="32" max="32" width="34.44140625" customWidth="true" bestFit="true" hidden="true"/>
     <col min="33" max="33" width="9.046875" customWidth="true" bestFit="true" hidden="true"/>
     <col min="34" max="34" width="9.46484375" customWidth="true" bestFit="true"/>
     <col min="35" max="35" width="100.703125" customWidth="true"/>
@@ -1101,13 +1148,13 @@
         <v>73</v>
       </c>
       <c r="K5" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="L5" t="s" s="2">
         <v>88</v>
       </c>
-      <c r="L5" t="s" s="2">
-        <v>89</v>
-      </c>
       <c r="M5" t="s" s="2">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="N5" s="2"/>
       <c r="O5" s="2"/>
@@ -1158,7 +1205,7 @@
         <v>73</v>
       </c>
       <c r="AF5" t="s" s="2">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="AG5" t="s" s="2">
         <v>79</v>
@@ -1175,10 +1222,10 @@
     </row>
     <row r="6">
       <c r="A6" t="s" s="2">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B6" t="s" s="2">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" t="s" s="2">
@@ -1189,7 +1236,7 @@
         <v>74</v>
       </c>
       <c r="G6" t="s" s="2">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="H6" t="s" s="2">
         <v>73</v>
@@ -1201,13 +1248,13 @@
         <v>73</v>
       </c>
       <c r="K6" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="L6" t="s" s="2">
         <v>92</v>
       </c>
-      <c r="L6" t="s" s="2">
-        <v>93</v>
-      </c>
       <c r="M6" t="s" s="2">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="N6" s="2"/>
       <c r="O6" s="2"/>
@@ -1258,7 +1305,7 @@
         <v>73</v>
       </c>
       <c r="AF6" t="s" s="2">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="AG6" t="s" s="2">
         <v>74</v>
@@ -1275,10 +1322,10 @@
     </row>
     <row r="7">
       <c r="A7" t="s" s="2">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B7" t="s" s="2">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" t="s" s="2">
@@ -1289,7 +1336,7 @@
         <v>74</v>
       </c>
       <c r="G7" t="s" s="2">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="H7" t="s" s="2">
         <v>73</v>
@@ -1301,7 +1348,7 @@
         <v>73</v>
       </c>
       <c r="K7" t="s" s="2">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="L7" t="s" s="2">
         <v>96</v>
@@ -1386,10 +1433,10 @@
       </c>
       <c r="E8" s="2"/>
       <c r="F8" t="s" s="2">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="G8" t="s" s="2">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="H8" t="s" s="2">
         <v>73</v>
@@ -1458,18 +1505,418 @@
         <v>73</v>
       </c>
       <c r="AF8" t="s" s="2">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="AG8" t="s" s="2">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="AH8" t="s" s="2">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="AI8" t="s" s="2">
         <v>73</v>
       </c>
       <c r="AJ8" t="s" s="2">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="2">
+        <v>102</v>
+      </c>
+      <c r="B9" t="s" s="2">
+        <v>102</v>
+      </c>
+      <c r="C9" s="2"/>
+      <c r="D9" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="E9" s="2"/>
+      <c r="F9" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="G9" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="H9" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="I9" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="J9" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="K9" t="s" s="2">
+        <v>103</v>
+      </c>
+      <c r="L9" t="s" s="2">
+        <v>104</v>
+      </c>
+      <c r="M9" t="s" s="2">
+        <v>104</v>
+      </c>
+      <c r="N9" s="2"/>
+      <c r="O9" s="2"/>
+      <c r="P9" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Q9" s="2"/>
+      <c r="R9" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="S9" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="T9" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="U9" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="V9" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="W9" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="X9" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Y9" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Z9" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AA9" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AB9" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AC9" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AD9" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AE9" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AF9" t="s" s="2">
+        <v>105</v>
+      </c>
+      <c r="AG9" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AH9" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AI9" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AJ9" t="s" s="2">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="2">
+        <v>106</v>
+      </c>
+      <c r="B10" t="s" s="2">
+        <v>106</v>
+      </c>
+      <c r="C10" s="2"/>
+      <c r="D10" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="E10" s="2"/>
+      <c r="F10" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="G10" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="H10" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="I10" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="J10" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="K10" t="s" s="2">
+        <v>107</v>
+      </c>
+      <c r="L10" t="s" s="2">
+        <v>108</v>
+      </c>
+      <c r="M10" t="s" s="2">
+        <v>108</v>
+      </c>
+      <c r="N10" s="2"/>
+      <c r="O10" s="2"/>
+      <c r="P10" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Q10" s="2"/>
+      <c r="R10" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="S10" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="T10" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="U10" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="V10" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="W10" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="X10" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Y10" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Z10" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AA10" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AB10" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AC10" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AD10" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AE10" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AF10" t="s" s="2">
+        <v>109</v>
+      </c>
+      <c r="AG10" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AH10" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AI10" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AJ10" t="s" s="2">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="2">
+        <v>110</v>
+      </c>
+      <c r="B11" t="s" s="2">
+        <v>110</v>
+      </c>
+      <c r="C11" s="2"/>
+      <c r="D11" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="E11" s="2"/>
+      <c r="F11" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="G11" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="H11" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="I11" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="J11" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="K11" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="L11" t="s" s="2">
+        <v>111</v>
+      </c>
+      <c r="M11" t="s" s="2">
+        <v>111</v>
+      </c>
+      <c r="N11" s="2"/>
+      <c r="O11" s="2"/>
+      <c r="P11" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Q11" s="2"/>
+      <c r="R11" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="S11" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="T11" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="U11" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="V11" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="W11" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="X11" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Y11" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Z11" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AA11" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AB11" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AC11" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AD11" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AE11" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AF11" t="s" s="2">
+        <v>112</v>
+      </c>
+      <c r="AG11" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AH11" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AI11" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AJ11" t="s" s="2">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s" s="2">
+        <v>113</v>
+      </c>
+      <c r="B12" t="s" s="2">
+        <v>113</v>
+      </c>
+      <c r="C12" s="2"/>
+      <c r="D12" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="E12" s="2"/>
+      <c r="F12" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="G12" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="H12" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="I12" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="J12" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="K12" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="L12" t="s" s="2">
+        <v>114</v>
+      </c>
+      <c r="M12" t="s" s="2">
+        <v>114</v>
+      </c>
+      <c r="N12" s="2"/>
+      <c r="O12" s="2"/>
+      <c r="P12" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Q12" s="2"/>
+      <c r="R12" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="S12" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="T12" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="U12" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="V12" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="W12" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="X12" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Y12" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Z12" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AA12" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AB12" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AC12" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AD12" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AE12" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AF12" t="s" s="2">
+        <v>115</v>
+      </c>
+      <c r="AG12" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AH12" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AI12" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AJ12" t="s" s="2">
         <v>73</v>
       </c>
     </row>

</xml_diff>